<commit_message>
Update backtest report for 2026-04-08
</commit_message>
<xml_diff>
--- a/backtest_report.xlsx
+++ b/backtest_report.xlsx
@@ -486,7 +486,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Son Güncelleme: 2026-04-08 08:59</t>
+          <t>Son Güncelleme: 2026-04-08 15:16</t>
         </is>
       </c>
     </row>
@@ -928,7 +928,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Son Güncelleme: 2026-04-08 08:59</t>
+          <t>Son Güncelleme: 2026-04-08 15:16</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update backtest report for 2026-04-09
</commit_message>
<xml_diff>
--- a/backtest_report.xlsx
+++ b/backtest_report.xlsx
@@ -47,14 +47,14 @@
       <sz val="10"/>
     </font>
     <font>
-      <color rgb="009C0006"/>
+      <color rgb="00006100"/>
     </font>
     <font>
       <b val="1"/>
       <color rgb="000070C0"/>
     </font>
     <font>
-      <color rgb="00006100"/>
+      <color rgb="009C0006"/>
     </font>
   </fonts>
   <fills count="3">
@@ -486,7 +486,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Son Güncelleme: 2026-04-08 17:08</t>
+          <t>Son Güncelleme: 2026-04-09 07:32</t>
         </is>
       </c>
     </row>
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>-0.02%</t>
+          <t>0.39%</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -574,7 +574,7 @@
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>0.29%</t>
+          <t>0.61%</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -584,7 +584,7 @@
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>-0.46%</t>
+          <t>-0.01%</t>
         </is>
       </c>
     </row>
@@ -664,20 +664,20 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="F8" t="n">
         <v>9.012700000000001</v>
       </c>
       <c r="G8" t="n">
-        <v>8.971500000000001</v>
+        <v>9.0639</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>-0.46</v>
+        <v>0.57</v>
       </c>
       <c r="I8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J8" s="7" t="inlineStr">
         <is>
@@ -705,20 +705,20 @@
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="F9" t="n">
         <v>45.2262</v>
       </c>
       <c r="G9" t="n">
-        <v>45.198</v>
+        <v>45.479</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>-0.06</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="I9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J9" s="7" t="inlineStr">
         <is>
@@ -746,20 +746,20 @@
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="F10" t="n">
         <v>47.7474</v>
       </c>
       <c r="G10" t="n">
-        <v>47.8027</v>
-      </c>
-      <c r="H10" s="8" t="n">
-        <v>0.12</v>
+        <v>47.9039</v>
+      </c>
+      <c r="H10" s="6" t="n">
+        <v>0.33</v>
       </c>
       <c r="I10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J10" s="7" t="inlineStr">
         <is>
@@ -796,7 +796,7 @@
       <c r="G11" t="n">
         <v>9.7357</v>
       </c>
-      <c r="H11" s="8" t="n">
+      <c r="H11" s="6" t="n">
         <v>0.29</v>
       </c>
       <c r="I11" t="n">
@@ -828,20 +828,20 @@
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="F12" t="n">
         <v>1.8861</v>
       </c>
       <c r="G12" t="n">
-        <v>1.8861</v>
-      </c>
-      <c r="H12" s="6" t="n">
-        <v>0</v>
+        <v>1.886</v>
+      </c>
+      <c r="H12" s="8" t="n">
+        <v>-0.01</v>
       </c>
       <c r="I12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J12" s="7" t="inlineStr">
         <is>
@@ -869,20 +869,20 @@
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="F13" t="n">
         <v>59.7798</v>
       </c>
       <c r="G13" t="n">
-        <v>59.7798</v>
+        <v>60.146</v>
       </c>
       <c r="H13" s="6" t="n">
-        <v>0</v>
+        <v>0.61</v>
       </c>
       <c r="I13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J13" s="7" t="inlineStr">
         <is>
@@ -902,7 +902,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K36"/>
+  <dimension ref="A1:K37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -928,7 +928,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Son Güncelleme: 2026-04-08 17:08</t>
+          <t>Son Güncelleme: 2026-04-09 07:32</t>
         </is>
       </c>
     </row>
@@ -939,7 +939,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -947,7 +947,7 @@
         </is>
       </c>
       <c r="D4" s="4" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
@@ -986,7 +986,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>0.3%</t>
+          <t>1.35%</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -1016,7 +1016,7 @@
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>2.32%</t>
+          <t>6.01%</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -1026,7 +1026,7 @@
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>-3.99%</t>
+          <t>-3.42%</t>
         </is>
       </c>
     </row>
@@ -1106,20 +1106,20 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="F8" t="n">
         <v>49.2657</v>
       </c>
       <c r="G8" t="n">
-        <v>47.2977</v>
-      </c>
-      <c r="H8" s="6" t="n">
-        <v>-3.99</v>
+        <v>47.5787</v>
+      </c>
+      <c r="H8" s="8" t="n">
+        <v>-3.42</v>
       </c>
       <c r="I8" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J8" s="7" t="inlineStr">
         <is>
@@ -1147,20 +1147,20 @@
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="F9" t="n">
         <v>14.7646</v>
       </c>
       <c r="G9" t="n">
-        <v>14.9393</v>
-      </c>
-      <c r="H9" s="8" t="n">
-        <v>1.18</v>
+        <v>15.1655</v>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>2.72</v>
       </c>
       <c r="I9" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J9" s="7" t="inlineStr">
         <is>
@@ -1188,20 +1188,20 @@
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="F10" t="n">
         <v>1.8046</v>
       </c>
       <c r="G10" t="n">
-        <v>1.7571</v>
+        <v>1.8149</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>-2.63</v>
+        <v>0.57</v>
       </c>
       <c r="I10" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J10" s="7" t="inlineStr">
         <is>
@@ -1229,20 +1229,20 @@
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="F11" t="n">
         <v>5.7386</v>
       </c>
       <c r="G11" t="n">
-        <v>5.7222</v>
+        <v>5.9405</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>-0.29</v>
+        <v>3.52</v>
       </c>
       <c r="I11" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="J11" s="7" t="inlineStr">
         <is>
@@ -1270,20 +1270,20 @@
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="F12" t="n">
         <v>1.1033</v>
       </c>
       <c r="G12" t="n">
-        <v>1.1113</v>
-      </c>
-      <c r="H12" s="8" t="n">
-        <v>0.73</v>
+        <v>1.1307</v>
+      </c>
+      <c r="H12" s="6" t="n">
+        <v>2.48</v>
       </c>
       <c r="I12" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J12" s="7" t="inlineStr">
         <is>
@@ -1311,20 +1311,20 @@
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="F13" t="n">
         <v>1.3449</v>
       </c>
       <c r="G13" t="n">
-        <v>1.3516</v>
-      </c>
-      <c r="H13" s="8" t="n">
-        <v>0.5</v>
+        <v>1.4022</v>
+      </c>
+      <c r="H13" s="6" t="n">
+        <v>4.26</v>
       </c>
       <c r="I13" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J13" s="7" t="inlineStr">
         <is>
@@ -1352,20 +1352,20 @@
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="F14" t="n">
         <v>43.6209</v>
       </c>
       <c r="G14" t="n">
-        <v>44.08</v>
-      </c>
-      <c r="H14" s="8" t="n">
-        <v>1.05</v>
+        <v>44.0006</v>
+      </c>
+      <c r="H14" s="6" t="n">
+        <v>0.87</v>
       </c>
       <c r="I14" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J14" s="7" t="inlineStr">
         <is>
@@ -1393,20 +1393,20 @@
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="F15" t="n">
         <v>1.1435</v>
       </c>
       <c r="G15" t="n">
-        <v>1.17</v>
-      </c>
-      <c r="H15" s="8" t="n">
-        <v>2.32</v>
+        <v>1.2122</v>
+      </c>
+      <c r="H15" s="6" t="n">
+        <v>6.01</v>
       </c>
       <c r="I15" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="J15" s="7" t="inlineStr">
         <is>
@@ -1434,20 +1434,20 @@
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="F16" t="n">
         <v>1.3849</v>
       </c>
       <c r="G16" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="H16" s="8" t="n">
-        <v>1.09</v>
+        <v>1.4058</v>
+      </c>
+      <c r="H16" s="6" t="n">
+        <v>1.51</v>
       </c>
       <c r="I16" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="J16" s="7" t="inlineStr">
         <is>
@@ -1475,20 +1475,20 @@
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="F17" t="n">
         <v>6.4409</v>
       </c>
       <c r="G17" t="n">
-        <v>6.5881</v>
-      </c>
-      <c r="H17" s="8" t="n">
-        <v>2.29</v>
+        <v>6.5702</v>
+      </c>
+      <c r="H17" s="6" t="n">
+        <v>2.01</v>
       </c>
       <c r="I17" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="J17" s="7" t="inlineStr">
         <is>
@@ -1516,20 +1516,20 @@
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="F18" t="n">
         <v>1.418</v>
       </c>
       <c r="G18" t="n">
-        <v>1.4042</v>
+        <v>1.4496</v>
       </c>
       <c r="H18" s="6" t="n">
-        <v>-0.97</v>
+        <v>2.23</v>
       </c>
       <c r="I18" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J18" s="7" t="inlineStr">
         <is>
@@ -1557,20 +1557,20 @@
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="F19" t="n">
         <v>45.5118</v>
       </c>
       <c r="G19" t="n">
-        <v>45.779</v>
-      </c>
-      <c r="H19" s="8" t="n">
-        <v>0.59</v>
+        <v>45.7548</v>
+      </c>
+      <c r="H19" s="6" t="n">
+        <v>0.53</v>
       </c>
       <c r="I19" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J19" s="7" t="inlineStr">
         <is>
@@ -1598,20 +1598,20 @@
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="F20" t="n">
         <v>11.1299</v>
       </c>
       <c r="G20" t="n">
-        <v>11.2665</v>
-      </c>
-      <c r="H20" s="8" t="n">
-        <v>1.23</v>
+        <v>11.2863</v>
+      </c>
+      <c r="H20" s="6" t="n">
+        <v>1.41</v>
       </c>
       <c r="I20" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J20" s="7" t="inlineStr">
         <is>
@@ -1639,20 +1639,20 @@
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="F21" t="n">
         <v>0.8579</v>
       </c>
       <c r="G21" t="n">
-        <v>0.8546</v>
-      </c>
-      <c r="H21" s="6" t="n">
-        <v>-0.38</v>
+        <v>0.8556</v>
+      </c>
+      <c r="H21" s="8" t="n">
+        <v>-0.27</v>
       </c>
       <c r="I21" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J21" s="7" t="inlineStr">
         <is>
@@ -1680,20 +1680,20 @@
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="F22" t="n">
         <v>9.3819</v>
       </c>
       <c r="G22" t="n">
-        <v>9.5289</v>
-      </c>
-      <c r="H22" s="8" t="n">
-        <v>1.57</v>
+        <v>9.5383</v>
+      </c>
+      <c r="H22" s="6" t="n">
+        <v>1.67</v>
       </c>
       <c r="I22" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J22" s="7" t="inlineStr">
         <is>
@@ -1721,20 +1721,20 @@
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="F23" t="n">
         <v>1.447</v>
       </c>
       <c r="G23" t="n">
-        <v>1.4578</v>
-      </c>
-      <c r="H23" s="8" t="n">
-        <v>0.75</v>
+        <v>1.4581</v>
+      </c>
+      <c r="H23" s="6" t="n">
+        <v>0.77</v>
       </c>
       <c r="I23" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="J23" s="7" t="inlineStr">
         <is>
@@ -1762,20 +1762,20 @@
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="F24" t="n">
         <v>44.6737</v>
       </c>
       <c r="G24" t="n">
-        <v>44.8884</v>
-      </c>
-      <c r="H24" s="8" t="n">
-        <v>0.48</v>
+        <v>44.8251</v>
+      </c>
+      <c r="H24" s="6" t="n">
+        <v>0.34</v>
       </c>
       <c r="I24" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="J24" s="7" t="inlineStr">
         <is>
@@ -1803,20 +1803,20 @@
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="F25" t="n">
         <v>4.8962</v>
       </c>
       <c r="G25" t="n">
-        <v>4.9885</v>
-      </c>
-      <c r="H25" s="8" t="n">
-        <v>1.89</v>
+        <v>4.9831</v>
+      </c>
+      <c r="H25" s="6" t="n">
+        <v>1.77</v>
       </c>
       <c r="I25" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="J25" s="7" t="inlineStr">
         <is>
@@ -1844,20 +1844,20 @@
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="F26" t="n">
         <v>53.0875</v>
       </c>
       <c r="G26" t="n">
-        <v>53.2566</v>
-      </c>
-      <c r="H26" s="8" t="n">
-        <v>0.32</v>
+        <v>53.8052</v>
+      </c>
+      <c r="H26" s="6" t="n">
+        <v>1.35</v>
       </c>
       <c r="I26" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J26" s="7" t="inlineStr">
         <is>
@@ -1885,20 +1885,20 @@
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="F27" t="n">
         <v>51.8381</v>
       </c>
       <c r="G27" t="n">
-        <v>51.9744</v>
-      </c>
-      <c r="H27" s="8" t="n">
-        <v>0.26</v>
+        <v>52.4948</v>
+      </c>
+      <c r="H27" s="6" t="n">
+        <v>1.27</v>
       </c>
       <c r="I27" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J27" s="7" t="inlineStr">
         <is>
@@ -1926,20 +1926,20 @@
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="F28" t="n">
         <v>9.022500000000001</v>
       </c>
       <c r="G28" t="n">
-        <v>8.971500000000001</v>
+        <v>9.0639</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-0.57</v>
+        <v>0.46</v>
       </c>
       <c r="I28" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J28" s="7" t="inlineStr">
         <is>
@@ -1967,20 +1967,20 @@
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="F29" t="n">
         <v>47.5867</v>
       </c>
       <c r="G29" t="n">
-        <v>47.8027</v>
-      </c>
-      <c r="H29" s="8" t="n">
-        <v>0.45</v>
+        <v>47.9039</v>
+      </c>
+      <c r="H29" s="6" t="n">
+        <v>0.67</v>
       </c>
       <c r="I29" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J29" s="7" t="inlineStr">
         <is>
@@ -2008,20 +2008,20 @@
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="F30" t="n">
         <v>1.6382</v>
       </c>
       <c r="G30" t="n">
-        <v>1.6388</v>
-      </c>
-      <c r="H30" s="8" t="n">
-        <v>0.04</v>
+        <v>1.6769</v>
+      </c>
+      <c r="H30" s="6" t="n">
+        <v>2.36</v>
       </c>
       <c r="I30" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J30" s="7" t="inlineStr">
         <is>
@@ -2049,20 +2049,20 @@
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="F31" t="n">
         <v>6.1635</v>
       </c>
       <c r="G31" t="n">
-        <v>6.2034</v>
-      </c>
-      <c r="H31" s="8" t="n">
-        <v>0.65</v>
+        <v>6.239</v>
+      </c>
+      <c r="H31" s="6" t="n">
+        <v>1.22</v>
       </c>
       <c r="I31" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J31" s="7" t="inlineStr">
         <is>
@@ -2090,20 +2090,20 @@
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="F32" t="n">
         <v>45.2262</v>
       </c>
       <c r="G32" t="n">
-        <v>45.198</v>
+        <v>45.479</v>
       </c>
       <c r="H32" s="6" t="n">
-        <v>-0.06</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="I32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J32" s="7" t="inlineStr">
         <is>
@@ -2140,7 +2140,7 @@
       <c r="G33" t="n">
         <v>9.7357</v>
       </c>
-      <c r="H33" s="8" t="n">
+      <c r="H33" s="6" t="n">
         <v>0.29</v>
       </c>
       <c r="I33" t="n">
@@ -2172,20 +2172,20 @@
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="F34" t="n">
         <v>59.7798</v>
       </c>
       <c r="G34" t="n">
-        <v>59.7798</v>
+        <v>60.146</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>0</v>
+        <v>0.61</v>
       </c>
       <c r="I34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J34" s="7" t="inlineStr">
         <is>
@@ -2213,20 +2213,20 @@
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="F35" t="n">
         <v>1.8861</v>
       </c>
       <c r="G35" t="n">
-        <v>1.8861</v>
-      </c>
-      <c r="H35" s="6" t="n">
-        <v>0</v>
+        <v>1.886</v>
+      </c>
+      <c r="H35" s="8" t="n">
+        <v>-0.01</v>
       </c>
       <c r="I35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J35" s="7" t="inlineStr">
         <is>
@@ -2254,27 +2254,68 @@
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="F36" t="n">
         <v>0.9747</v>
       </c>
       <c r="G36" t="n">
-        <v>0.9747</v>
+        <v>1</v>
       </c>
       <c r="H36" s="6" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="I36" t="n">
+        <v>1</v>
+      </c>
+      <c r="J36" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>YPN</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>61.8354</v>
+      </c>
+      <c r="G37" t="n">
+        <v>61.8354</v>
+      </c>
+      <c r="H37" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="I36" t="n">
+      <c r="I37" t="n">
         <v>0</v>
       </c>
-      <c r="J36" s="7" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="K36" t="inlineStr"/>
+      <c r="J37" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update backtest report for 2026-04-10
</commit_message>
<xml_diff>
--- a/backtest_report.xlsx
+++ b/backtest_report.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:K15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -486,7 +486,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Son Güncelleme: 2026-04-09 09:37</t>
+          <t>Son Güncelleme: 2026-04-10 07:05</t>
         </is>
       </c>
     </row>
@@ -497,7 +497,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -505,7 +505,7 @@
         </is>
       </c>
       <c r="D4" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>0.85%</t>
+          <t>0.76%</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -574,7 +574,7 @@
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>2.84%</t>
+          <t>2.88%</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -584,7 +584,7 @@
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>0.21%</t>
+          <t>0.0%</t>
         </is>
       </c>
     </row>
@@ -664,20 +664,20 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="F8" t="n">
         <v>9.012700000000001</v>
       </c>
       <c r="G8" t="n">
-        <v>9.0639</v>
+        <v>9.087899999999999</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>0.57</v>
+        <v>0.83</v>
       </c>
       <c r="I8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J8" s="7" t="inlineStr">
         <is>
@@ -705,20 +705,20 @@
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="F9" t="n">
         <v>45.2262</v>
       </c>
       <c r="G9" t="n">
-        <v>45.479</v>
+        <v>45.5477</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.71</v>
       </c>
       <c r="I9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J9" s="7" t="inlineStr">
         <is>
@@ -746,20 +746,20 @@
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="F10" t="n">
         <v>47.7474</v>
       </c>
       <c r="G10" t="n">
-        <v>47.9039</v>
+        <v>48.0258</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>0.33</v>
+        <v>0.58</v>
       </c>
       <c r="I10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J10" s="7" t="inlineStr">
         <is>
@@ -828,20 +828,20 @@
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="F12" t="n">
         <v>1.8861</v>
       </c>
       <c r="G12" t="n">
-        <v>1.9396</v>
+        <v>1.9404</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>2.84</v>
+        <v>2.88</v>
       </c>
       <c r="I12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J12" s="7" t="inlineStr">
         <is>
@@ -869,20 +869,20 @@
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="F13" t="n">
         <v>59.7798</v>
       </c>
       <c r="G13" t="n">
-        <v>60.146</v>
+        <v>60.277</v>
       </c>
       <c r="H13" s="6" t="n">
-        <v>0.61</v>
+        <v>0.83</v>
       </c>
       <c r="I13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J13" s="7" t="inlineStr">
         <is>
@@ -890,6 +890,88 @@
         </is>
       </c>
       <c r="K13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>HNS</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>45.9362</v>
+      </c>
+      <c r="G14" t="n">
+        <v>45.9362</v>
+      </c>
+      <c r="H14" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>IOH</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>48.1981</v>
+      </c>
+      <c r="G15" t="n">
+        <v>48.1981</v>
+      </c>
+      <c r="H15" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -902,7 +984,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K37"/>
+  <dimension ref="A1:K40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -928,7 +1010,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Son Güncelleme: 2026-04-09 09:37</t>
+          <t>Son Güncelleme: 2026-04-10 07:05</t>
         </is>
       </c>
     </row>
@@ -939,7 +1021,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -947,7 +1029,7 @@
         </is>
       </c>
       <c r="D4" s="4" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
@@ -986,7 +1068,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>1.45%</t>
+          <t>1.67%</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -1016,7 +1098,7 @@
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>6.01%</t>
+          <t>6.52%</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -1026,7 +1108,7 @@
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>-3.42%</t>
+          <t>-3.14%</t>
         </is>
       </c>
     </row>
@@ -1106,20 +1188,20 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="F8" t="n">
         <v>49.2657</v>
       </c>
       <c r="G8" t="n">
-        <v>47.5787</v>
+        <v>47.7169</v>
       </c>
       <c r="H8" s="8" t="n">
-        <v>-3.42</v>
+        <v>-3.14</v>
       </c>
       <c r="I8" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="J8" s="7" t="inlineStr">
         <is>
@@ -1147,20 +1229,20 @@
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="F9" t="n">
         <v>14.7646</v>
       </c>
       <c r="G9" t="n">
-        <v>15.1655</v>
+        <v>15.1583</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>2.72</v>
+        <v>2.67</v>
       </c>
       <c r="I9" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J9" s="7" t="inlineStr">
         <is>
@@ -1188,20 +1270,20 @@
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="F10" t="n">
         <v>1.8046</v>
       </c>
       <c r="G10" t="n">
-        <v>1.8149</v>
+        <v>1.8246</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>0.57</v>
+        <v>1.11</v>
       </c>
       <c r="I10" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J10" s="7" t="inlineStr">
         <is>
@@ -1229,20 +1311,20 @@
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="F11" t="n">
         <v>5.7386</v>
       </c>
       <c r="G11" t="n">
-        <v>5.9405</v>
+        <v>5.9995</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>3.52</v>
+        <v>4.55</v>
       </c>
       <c r="I11" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J11" s="7" t="inlineStr">
         <is>
@@ -1270,20 +1352,20 @@
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="F12" t="n">
         <v>1.1033</v>
       </c>
       <c r="G12" t="n">
-        <v>1.1307</v>
+        <v>1.1362</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>2.48</v>
+        <v>2.98</v>
       </c>
       <c r="I12" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J12" s="7" t="inlineStr">
         <is>
@@ -1311,20 +1393,20 @@
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="F13" t="n">
         <v>1.3449</v>
       </c>
       <c r="G13" t="n">
-        <v>1.4022</v>
+        <v>1.4224</v>
       </c>
       <c r="H13" s="6" t="n">
-        <v>4.26</v>
+        <v>5.76</v>
       </c>
       <c r="I13" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J13" s="7" t="inlineStr">
         <is>
@@ -1352,20 +1434,20 @@
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="F14" t="n">
         <v>43.6209</v>
       </c>
       <c r="G14" t="n">
-        <v>44.0006</v>
+        <v>44.4386</v>
       </c>
       <c r="H14" s="6" t="n">
-        <v>0.87</v>
+        <v>1.87</v>
       </c>
       <c r="I14" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J14" s="7" t="inlineStr">
         <is>
@@ -1393,20 +1475,20 @@
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="F15" t="n">
         <v>1.1435</v>
       </c>
       <c r="G15" t="n">
-        <v>1.2122</v>
+        <v>1.2181</v>
       </c>
       <c r="H15" s="6" t="n">
-        <v>6.01</v>
+        <v>6.52</v>
       </c>
       <c r="I15" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J15" s="7" t="inlineStr">
         <is>
@@ -1434,20 +1516,20 @@
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="F16" t="n">
         <v>1.3849</v>
       </c>
       <c r="G16" t="n">
-        <v>1.4058</v>
+        <v>1.4282</v>
       </c>
       <c r="H16" s="6" t="n">
-        <v>1.51</v>
+        <v>3.13</v>
       </c>
       <c r="I16" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J16" s="7" t="inlineStr">
         <is>
@@ -1475,20 +1557,20 @@
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="F17" t="n">
         <v>6.4409</v>
       </c>
       <c r="G17" t="n">
-        <v>6.5702</v>
+        <v>6.6176</v>
       </c>
       <c r="H17" s="6" t="n">
-        <v>2.01</v>
+        <v>2.74</v>
       </c>
       <c r="I17" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J17" s="7" t="inlineStr">
         <is>
@@ -1516,20 +1598,20 @@
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="F18" t="n">
         <v>1.418</v>
       </c>
       <c r="G18" t="n">
-        <v>1.4496</v>
+        <v>1.458</v>
       </c>
       <c r="H18" s="6" t="n">
-        <v>2.23</v>
+        <v>2.82</v>
       </c>
       <c r="I18" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="J18" s="7" t="inlineStr">
         <is>
@@ -1557,20 +1639,20 @@
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="F19" t="n">
         <v>45.5118</v>
       </c>
       <c r="G19" t="n">
-        <v>45.7548</v>
+        <v>45.8137</v>
       </c>
       <c r="H19" s="6" t="n">
-        <v>0.53</v>
+        <v>0.66</v>
       </c>
       <c r="I19" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="J19" s="7" t="inlineStr">
         <is>
@@ -1598,20 +1680,20 @@
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="F20" t="n">
         <v>11.1299</v>
       </c>
       <c r="G20" t="n">
-        <v>11.2863</v>
+        <v>11.3034</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>1.41</v>
+        <v>1.56</v>
       </c>
       <c r="I20" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J20" s="7" t="inlineStr">
         <is>
@@ -1639,20 +1721,20 @@
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="F21" t="n">
         <v>0.8579</v>
       </c>
       <c r="G21" t="n">
-        <v>0.8556</v>
-      </c>
-      <c r="H21" s="8" t="n">
-        <v>-0.27</v>
+        <v>0.8605</v>
+      </c>
+      <c r="H21" s="6" t="n">
+        <v>0.3</v>
       </c>
       <c r="I21" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J21" s="7" t="inlineStr">
         <is>
@@ -1680,20 +1762,20 @@
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="F22" t="n">
         <v>9.3819</v>
       </c>
       <c r="G22" t="n">
-        <v>9.5383</v>
+        <v>9.5481</v>
       </c>
       <c r="H22" s="6" t="n">
-        <v>1.67</v>
+        <v>1.77</v>
       </c>
       <c r="I22" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J22" s="7" t="inlineStr">
         <is>
@@ -1721,20 +1803,20 @@
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="F23" t="n">
         <v>1.447</v>
       </c>
       <c r="G23" t="n">
-        <v>1.4581</v>
+        <v>1.46</v>
       </c>
       <c r="H23" s="6" t="n">
-        <v>0.77</v>
+        <v>0.9</v>
       </c>
       <c r="I23" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J23" s="7" t="inlineStr">
         <is>
@@ -1762,20 +1844,20 @@
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="F24" t="n">
         <v>44.6737</v>
       </c>
       <c r="G24" t="n">
-        <v>44.8251</v>
+        <v>44.8929</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>0.34</v>
+        <v>0.49</v>
       </c>
       <c r="I24" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J24" s="7" t="inlineStr">
         <is>
@@ -1803,20 +1885,20 @@
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="F25" t="n">
         <v>4.8962</v>
       </c>
       <c r="G25" t="n">
-        <v>4.9957</v>
+        <v>5.0255</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>2.03</v>
+        <v>2.64</v>
       </c>
       <c r="I25" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J25" s="7" t="inlineStr">
         <is>
@@ -1844,20 +1926,20 @@
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="F26" t="n">
         <v>53.0875</v>
       </c>
       <c r="G26" t="n">
-        <v>53.8052</v>
+        <v>53.7924</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>1.35</v>
+        <v>1.33</v>
       </c>
       <c r="I26" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="J26" s="7" t="inlineStr">
         <is>
@@ -1885,20 +1967,20 @@
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="F27" t="n">
         <v>51.8381</v>
       </c>
       <c r="G27" t="n">
-        <v>52.4948</v>
+        <v>52.4846</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>1.27</v>
+        <v>1.25</v>
       </c>
       <c r="I27" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="J27" s="7" t="inlineStr">
         <is>
@@ -1926,20 +2008,20 @@
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="F28" t="n">
         <v>9.022500000000001</v>
       </c>
       <c r="G28" t="n">
-        <v>9.0639</v>
+        <v>9.087899999999999</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>0.46</v>
+        <v>0.72</v>
       </c>
       <c r="I28" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J28" s="7" t="inlineStr">
         <is>
@@ -1967,20 +2049,20 @@
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="F29" t="n">
         <v>47.5867</v>
       </c>
       <c r="G29" t="n">
-        <v>47.9039</v>
+        <v>48.0258</v>
       </c>
       <c r="H29" s="6" t="n">
-        <v>0.67</v>
+        <v>0.92</v>
       </c>
       <c r="I29" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J29" s="7" t="inlineStr">
         <is>
@@ -2008,20 +2090,20 @@
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="F30" t="n">
         <v>1.6382</v>
       </c>
       <c r="G30" t="n">
-        <v>1.6769</v>
+        <v>1.6814</v>
       </c>
       <c r="H30" s="6" t="n">
-        <v>2.36</v>
+        <v>2.64</v>
       </c>
       <c r="I30" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J30" s="7" t="inlineStr">
         <is>
@@ -2049,20 +2131,20 @@
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="F31" t="n">
         <v>6.1635</v>
       </c>
       <c r="G31" t="n">
-        <v>6.239</v>
+        <v>6.253</v>
       </c>
       <c r="H31" s="6" t="n">
-        <v>1.22</v>
+        <v>1.45</v>
       </c>
       <c r="I31" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J31" s="7" t="inlineStr">
         <is>
@@ -2090,20 +2172,20 @@
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="F32" t="n">
         <v>45.2262</v>
       </c>
       <c r="G32" t="n">
-        <v>45.479</v>
+        <v>45.5477</v>
       </c>
       <c r="H32" s="6" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.71</v>
       </c>
       <c r="I32" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J32" s="7" t="inlineStr">
         <is>
@@ -2172,20 +2254,20 @@
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="F34" t="n">
         <v>59.7798</v>
       </c>
       <c r="G34" t="n">
-        <v>60.146</v>
+        <v>60.277</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>0.61</v>
+        <v>0.83</v>
       </c>
       <c r="I34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J34" s="7" t="inlineStr">
         <is>
@@ -2213,20 +2295,20 @@
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="F35" t="n">
         <v>1.8861</v>
       </c>
       <c r="G35" t="n">
-        <v>1.9396</v>
+        <v>1.9404</v>
       </c>
       <c r="H35" s="6" t="n">
-        <v>2.84</v>
+        <v>2.88</v>
       </c>
       <c r="I35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J35" s="7" t="inlineStr">
         <is>
@@ -2254,20 +2336,20 @@
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="F36" t="n">
         <v>0.9747</v>
       </c>
       <c r="G36" t="n">
-        <v>1</v>
+        <v>1.0048</v>
       </c>
       <c r="H36" s="6" t="n">
-        <v>2.6</v>
+        <v>3.09</v>
       </c>
       <c r="I36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J36" s="7" t="inlineStr">
         <is>
@@ -2295,27 +2377,150 @@
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="F37" t="n">
         <v>61.8354</v>
       </c>
       <c r="G37" t="n">
-        <v>61.8354</v>
+        <v>61.7754</v>
       </c>
       <c r="H37" s="8" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="I37" t="n">
+        <v>1</v>
+      </c>
+      <c r="J37" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>IOH</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>48.1981</v>
+      </c>
+      <c r="G38" t="n">
+        <v>48.1981</v>
+      </c>
+      <c r="H38" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="I37" t="n">
+      <c r="I38" t="n">
         <v>0</v>
       </c>
-      <c r="J37" s="7" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="K37" t="inlineStr"/>
+      <c r="J38" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>HNS</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>45.9362</v>
+      </c>
+      <c r="G39" t="n">
+        <v>45.9362</v>
+      </c>
+      <c r="H39" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" t="n">
+        <v>0</v>
+      </c>
+      <c r="J39" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>BVK</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>1.0422</v>
+      </c>
+      <c r="G40" t="n">
+        <v>1.0422</v>
+      </c>
+      <c r="H40" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I40" t="n">
+        <v>0</v>
+      </c>
+      <c r="J40" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>